<commit_message>
fix: validate accounting inputs and preserve source evidence
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCBBE89-F138-4682-889B-232CFE7A1EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8179E1-E57C-47CA-B358-F58A103316F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -488,7 +488,7 @@
     <t>Experimental review aid. Not a Division 7A determination, not an ATO assessment, and not tax, legal or financial advice.</t>
   </si>
   <si>
-    <t>Excel 16.0 build 20326</t>
+    <t>Excel 16.0 build 20430</t>
   </si>
 </sst>
 </file>
@@ -729,10 +729,10 @@
       <calculatedColumnFormula>IF(AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),ISNUMBER(Summary!$B$3),Summary!$B$3&gt;0,ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&gt;0),ROUND(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]*Summary!$B$3/(1-(1/(1+Summary!$B$3))^tblLoans[[#This Row],[Term_used]]),2),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="MYR_verdict">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="MYR_reason">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="MYR_required">
       <calculatedColumnFormula>IF(OR(tblLoans[[#This Row],[MYR_verdict]]="MYR_MET",tblLoans[[#This Row],[MYR_verdict]]="MYR_SHORT"),tblLoans[[#This Row],[MYR_raw]],"")</calculatedColumnFormula>
@@ -1352,11 +1352,11 @@
         <v>47212.37</v>
       </c>
       <c r="AB2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>MYR_SHORT</v>
       </c>
       <c r="AC2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD2" s="10">
@@ -1480,11 +1480,11 @@
         <v>27640.06</v>
       </c>
       <c r="AB3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD3" s="10" t="str">
@@ -1608,11 +1608,11 @@
         <v>28334.799999999999</v>
       </c>
       <c r="AB4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is UNKNOWN, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD4" s="10" t="str">
@@ -1736,11 +1736,11 @@
         <v>22489.279999999999</v>
       </c>
       <c r="AB5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>UNKNOWN</v>
       </c>
       <c r="AC5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>payments applied not established</v>
       </c>
       <c r="AD5" s="10" t="str">
@@ -1864,11 +1864,11 @@
         <v/>
       </c>
       <c r="AB6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>nil remaining term under s 109E(6)</v>
       </c>
       <c r="AD6" s="10" t="str">
@@ -1992,11 +1992,11 @@
         <v>36713.81</v>
       </c>
       <c r="AB7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD7" s="10" t="str">
@@ -2122,11 +2122,11 @@
         <v/>
       </c>
       <c r="AB8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD8" s="10" t="str">
@@ -2250,11 +2250,11 @@
         <v/>
       </c>
       <c r="AB9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD9" s="10" t="str">

</xml_diff>

<commit_message>
fix: validate accounting inputs and preserve source evidence (#154)
Correct Division 7A year checks, pending payroll statuses and duplicate-payday allocation. Preserve source-byte provenance, reject invalid monetary inputs and require an explicit dividend payment date. Clarify the documented calculation scope.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCBBE89-F138-4682-889B-232CFE7A1EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8179E1-E57C-47CA-B358-F58A103316F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -488,7 +488,7 @@
     <t>Experimental review aid. Not a Division 7A determination, not an ATO assessment, and not tax, legal or financial advice.</t>
   </si>
   <si>
-    <t>Excel 16.0 build 20326</t>
+    <t>Excel 16.0 build 20430</t>
   </si>
 </sst>
 </file>
@@ -729,10 +729,10 @@
       <calculatedColumnFormula>IF(AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),ISNUMBER(Summary!$B$3),Summary!$B$3&gt;0,ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&gt;0),ROUND(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]*Summary!$B$3/(1-(1/(1+Summary!$B$3))^tblLoans[[#This Row],[Term_used]]),2),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="MYR_verdict">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="MYR_reason">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="MYR_required">
       <calculatedColumnFormula>IF(OR(tblLoans[[#This Row],[MYR_verdict]]="MYR_MET",tblLoans[[#This Row],[MYR_verdict]]="MYR_SHORT"),tblLoans[[#This Row],[MYR_raw]],"")</calculatedColumnFormula>
@@ -1352,11 +1352,11 @@
         <v>47212.37</v>
       </c>
       <c r="AB2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>MYR_SHORT</v>
       </c>
       <c r="AC2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD2" s="10">
@@ -1480,11 +1480,11 @@
         <v>27640.06</v>
       </c>
       <c r="AB3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD3" s="10" t="str">
@@ -1608,11 +1608,11 @@
         <v>28334.799999999999</v>
       </c>
       <c r="AB4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is UNKNOWN, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD4" s="10" t="str">
@@ -1736,11 +1736,11 @@
         <v>22489.279999999999</v>
       </c>
       <c r="AB5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>UNKNOWN</v>
       </c>
       <c r="AC5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>payments applied not established</v>
       </c>
       <c r="AD5" s="10" t="str">
@@ -1864,11 +1864,11 @@
         <v/>
       </c>
       <c r="AB6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>nil remaining term under s 109E(6)</v>
       </c>
       <c r="AD6" s="10" t="str">
@@ -1992,11 +1992,11 @@
         <v>36713.81</v>
       </c>
       <c r="AB7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD7" s="10" t="str">
@@ -2122,11 +2122,11 @@
         <v/>
       </c>
       <c r="AB8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD8" s="10" t="str">
@@ -2250,11 +2250,11 @@
         <v/>
       </c>
       <c r="AB9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate")))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established"))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD9" s="10" t="str">

</xml_diff>